<commit_message>
fix exam bug (22)
</commit_message>
<xml_diff>
--- a/StudyHub.Frontend/public/example.xlsx
+++ b/StudyHub.Frontend/public/example.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VKHOANG\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5783F80-4B47-4606-9284-8BC311FFE402}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F994BF5-137A-4FE4-BD05-4B9CF241AA0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{08F7A277-DBC5-441D-8A75-065BBD69C901}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
   <si>
     <t>Tên câu hỏi</t>
   </si>
@@ -102,6 +102,18 @@
   </si>
   <si>
     <t>đảo, chuồng</t>
+  </si>
+  <si>
+    <t>matching</t>
+  </si>
+  <si>
+    <t>Nối từ cho đúng</t>
+  </si>
+  <si>
+    <t>yêu cô giáo, đi câu cá</t>
+  </si>
+  <si>
+    <t>bố, bé</t>
   </si>
 </sst>
 </file>
@@ -465,7 +477,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CB38FAA-26FA-43A4-AEC3-B459A691ACE6}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -555,10 +567,24 @@
         <v>21</v>
       </c>
     </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A1048576" xr:uid="{465CE65B-7AAA-4195-AA7A-106A6F4A6411}">
-      <formula1>"single-choice, multiple-choice, text-input, fill-blank"</formula1>
+      <formula1>"single-choice, multiple-choice, text-input, fill-blank, matching"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Commit file after day 21/11
</commit_message>
<xml_diff>
--- a/StudyHub.Frontend/public/example.xlsx
+++ b/StudyHub.Frontend/public/example.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VKHOANG\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5783F80-4B47-4606-9284-8BC311FFE402}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F994BF5-137A-4FE4-BD05-4B9CF241AA0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{08F7A277-DBC5-441D-8A75-065BBD69C901}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
   <si>
     <t>Tên câu hỏi</t>
   </si>
@@ -102,6 +102,18 @@
   </si>
   <si>
     <t>đảo, chuồng</t>
+  </si>
+  <si>
+    <t>matching</t>
+  </si>
+  <si>
+    <t>Nối từ cho đúng</t>
+  </si>
+  <si>
+    <t>yêu cô giáo, đi câu cá</t>
+  </si>
+  <si>
+    <t>bố, bé</t>
   </si>
 </sst>
 </file>
@@ -465,7 +477,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CB38FAA-26FA-43A4-AEC3-B459A691ACE6}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -555,10 +567,24 @@
         <v>21</v>
       </c>
     </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A1048576" xr:uid="{465CE65B-7AAA-4195-AA7A-106A6F4A6411}">
-      <formula1>"single-choice, multiple-choice, text-input, fill-blank"</formula1>
+      <formula1>"single-choice, multiple-choice, text-input, fill-blank, matching"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>